<commit_message>
feat: filtros bairro, faixa de preço, banheiros, grupos
</commit_message>
<xml_diff>
--- a/VivaReal_Imoveis.xlsx
+++ b/VivaReal_Imoveis.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1556,7 +1556,7 @@
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1699,7 +1699,7 @@
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1848,7 +1848,7 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1944,7 +1944,7 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2034,7 +2034,7 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2083,7 +2083,7 @@
       <c r="B33" s="3" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2126,7 +2126,7 @@
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2175,7 +2175,7 @@
       <c r="B35" s="3" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2218,7 +2218,7 @@
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       <c r="B37" s="3" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2310,7 +2310,7 @@
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       <c r="B39" s="3" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2455,7 +2455,7 @@
       <c r="B41" s="3" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2498,7 +2498,7 @@
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2541,7 +2541,7 @@
       <c r="B43" s="3" t="inlineStr"/>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2637,7 +2637,7 @@
       <c r="B45" s="3" t="inlineStr"/>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       <c r="B47" s="3" t="inlineStr"/>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -2776,7 +2776,7 @@
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2866,7 +2866,7 @@
       <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2909,7 +2909,7 @@
       <c r="B51" s="3" t="inlineStr"/>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2952,7 +2952,7 @@
       <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -3001,7 +3001,7 @@
       <c r="B53" s="3" t="inlineStr"/>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -3050,7 +3050,7 @@
       <c r="B54" s="2" t="inlineStr"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -3152,7 +3152,7 @@
       <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -3195,7 +3195,7 @@
       <c r="B57" s="3" t="inlineStr"/>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -3244,7 +3244,7 @@
       <c r="B58" s="2" t="inlineStr"/>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3287,7 +3287,7 @@
       <c r="B59" s="3" t="inlineStr"/>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -3336,7 +3336,7 @@
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3383,7 +3383,7 @@
       <c r="B61" s="3" t="inlineStr"/>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3432,7 +3432,7 @@
       <c r="B62" s="2" t="inlineStr"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3481,7 +3481,7 @@
       <c r="B63" s="3" t="inlineStr"/>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3579,7 +3579,7 @@
       <c r="B65" s="3" t="inlineStr"/>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
       <c r="B66" s="2" t="inlineStr"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3671,7 +3671,7 @@
       <c r="B67" s="3" t="inlineStr"/>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -3720,7 +3720,7 @@
       <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -3816,7 +3816,7 @@
       <c r="B70" s="2" t="inlineStr"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3865,7 +3865,7 @@
       <c r="B71" s="3" t="inlineStr"/>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -3914,7 +3914,7 @@
       <c r="B72" s="2" t="inlineStr"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -4016,7 +4016,7 @@
       <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -4063,7 +4063,7 @@
       <c r="B75" s="3" t="inlineStr"/>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -4112,7 +4112,7 @@
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -4155,7 +4155,7 @@
       <c r="B77" s="3" t="inlineStr"/>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -4204,7 +4204,7 @@
       <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -4253,7 +4253,7 @@
       <c r="B79" s="3" t="inlineStr"/>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -4296,7 +4296,7 @@
       <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4345,7 +4345,7 @@
       <c r="B81" s="3" t="inlineStr"/>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4388,7 +4388,7 @@
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4431,7 +4431,7 @@
       <c r="B83" s="3" t="inlineStr"/>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -4474,7 +4474,7 @@
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
       <c r="B85" s="3" t="inlineStr"/>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4566,7 +4566,7 @@
       <c r="B86" s="2" t="inlineStr"/>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -4609,7 +4609,7 @@
       <c r="B87" s="3" t="inlineStr"/>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4652,7 +4652,7 @@
       <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4695,7 +4695,7 @@
       <c r="B89" s="3" t="inlineStr"/>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -4738,7 +4738,7 @@
       <c r="B90" s="2" t="inlineStr"/>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4781,7 +4781,7 @@
       <c r="B91" s="3" t="inlineStr"/>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4824,7 +4824,7 @@
       <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4863,7 +4863,7 @@
       <c r="B93" s="3" t="inlineStr"/>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -4912,7 +4912,7 @@
       <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4959,7 +4959,7 @@
       <c r="B95" s="3" t="inlineStr"/>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -5002,7 +5002,7 @@
       <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5051,7 +5051,7 @@
       <c r="B97" s="3" t="inlineStr"/>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -5094,7 +5094,7 @@
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5137,7 +5137,7 @@
       <c r="B99" s="3" t="inlineStr"/>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -5180,7 +5180,7 @@
       <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -5223,7 +5223,7 @@
       <c r="B101" s="3" t="inlineStr"/>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -5266,7 +5266,7 @@
       <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -5315,7 +5315,7 @@
       <c r="B103" s="3" t="inlineStr"/>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -5362,7 +5362,7 @@
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
       <c r="B105" s="3" t="inlineStr"/>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -5503,7 +5503,7 @@
       <c r="B107" s="3" t="inlineStr"/>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -5552,7 +5552,7 @@
       <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -5595,7 +5595,7 @@
       <c r="B109" s="3" t="inlineStr"/>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -5638,7 +5638,7 @@
       <c r="B110" s="2" t="inlineStr"/>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -5687,7 +5687,7 @@
       <c r="B111" s="3" t="inlineStr"/>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -5730,7 +5730,7 @@
       <c r="B112" s="2" t="inlineStr"/>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5773,7 +5773,7 @@
       <c r="B113" s="3" t="inlineStr"/>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -5822,7 +5822,7 @@
       <c r="B114" s="2" t="inlineStr"/>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="B115" s="3" t="inlineStr"/>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -5914,7 +5914,7 @@
       <c r="B116" s="2" t="inlineStr"/>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5963,7 +5963,7 @@
       <c r="B117" s="3" t="inlineStr"/>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -6012,7 +6012,7 @@
       <c r="B118" s="2" t="inlineStr"/>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -6061,7 +6061,7 @@
       <c r="B119" s="3" t="inlineStr"/>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -6104,7 +6104,7 @@
       <c r="B120" s="2" t="inlineStr"/>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -6151,7 +6151,7 @@
       <c r="B121" s="3" t="inlineStr"/>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -6194,7 +6194,7 @@
       <c r="B122" s="2" t="inlineStr"/>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -6243,7 +6243,7 @@
       <c r="B123" s="3" t="inlineStr"/>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -6292,7 +6292,7 @@
       <c r="B124" s="2" t="inlineStr"/>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -6335,7 +6335,7 @@
       <c r="B125" s="3" t="inlineStr"/>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -6384,7 +6384,7 @@
       <c r="B126" s="2" t="inlineStr"/>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -6433,7 +6433,7 @@
       <c r="B127" s="3" t="inlineStr"/>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -6482,7 +6482,7 @@
       <c r="B128" s="2" t="inlineStr"/>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -6525,7 +6525,7 @@
       <c r="B129" s="3" t="inlineStr"/>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -6568,7 +6568,7 @@
       <c r="B130" s="2" t="inlineStr"/>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -6611,7 +6611,7 @@
       <c r="B131" s="3" t="inlineStr"/>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -6654,7 +6654,7 @@
       <c r="B132" s="2" t="inlineStr"/>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -6703,7 +6703,7 @@
       <c r="B133" s="3" t="inlineStr"/>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -6750,7 +6750,7 @@
       <c r="B134" s="2" t="inlineStr"/>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -6799,7 +6799,7 @@
       <c r="B135" s="3" t="inlineStr"/>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -6848,7 +6848,7 @@
       <c r="B136" s="2" t="inlineStr"/>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6895,7 +6895,7 @@
       <c r="B137" s="3" t="inlineStr"/>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -6938,7 +6938,7 @@
       <c r="B138" s="2" t="inlineStr"/>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6987,7 +6987,7 @@
       <c r="B139" s="3" t="inlineStr"/>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -7030,7 +7030,7 @@
       <c r="B140" s="2" t="inlineStr"/>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -7073,7 +7073,7 @@
       <c r="B141" s="3" t="inlineStr"/>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -7122,7 +7122,7 @@
       <c r="B142" s="2" t="inlineStr"/>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -7171,7 +7171,7 @@
       <c r="B143" s="3" t="inlineStr"/>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -7220,7 +7220,7 @@
       <c r="B144" s="2" t="inlineStr"/>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -7269,7 +7269,7 @@
       <c r="B145" s="3" t="inlineStr"/>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -7312,7 +7312,7 @@
       <c r="B146" s="2" t="inlineStr"/>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -7355,7 +7355,7 @@
       <c r="B147" s="3" t="inlineStr"/>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -7404,7 +7404,7 @@
       <c r="B148" s="2" t="inlineStr"/>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -7447,7 +7447,7 @@
       <c r="B149" s="3" t="inlineStr"/>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -7496,7 +7496,7 @@
       <c r="B150" s="2" t="inlineStr"/>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -7539,7 +7539,7 @@
       <c r="B151" s="3" t="inlineStr"/>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -7582,7 +7582,7 @@
       <c r="B152" s="2" t="inlineStr"/>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -7631,7 +7631,7 @@
       <c r="B153" s="3" t="inlineStr"/>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -7680,7 +7680,7 @@
       <c r="B154" s="2" t="inlineStr"/>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -7723,7 +7723,7 @@
       <c r="B155" s="3" t="inlineStr"/>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -7772,7 +7772,7 @@
       <c r="B156" s="2" t="inlineStr"/>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -7815,7 +7815,7 @@
       <c r="B157" s="3" t="inlineStr"/>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -7864,7 +7864,7 @@
       <c r="B158" s="2" t="inlineStr"/>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -7913,7 +7913,7 @@
       <c r="B159" s="3" t="inlineStr"/>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -7962,7 +7962,7 @@
       <c r="B160" s="2" t="inlineStr"/>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -8005,7 +8005,7 @@
       <c r="B161" s="3" t="inlineStr"/>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -8048,7 +8048,7 @@
       <c r="B162" s="2" t="inlineStr"/>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -8097,7 +8097,7 @@
       <c r="B163" s="3" t="inlineStr"/>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -8146,7 +8146,7 @@
       <c r="B164" s="2" t="inlineStr"/>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -8189,7 +8189,7 @@
       <c r="B165" s="3" t="inlineStr"/>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -8232,7 +8232,7 @@
       <c r="B166" s="2" t="inlineStr"/>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -8275,7 +8275,7 @@
       <c r="B167" s="3" t="inlineStr"/>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -8324,7 +8324,7 @@
       <c r="B168" s="2" t="inlineStr"/>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -8373,7 +8373,7 @@
       <c r="B169" s="3" t="inlineStr"/>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -8420,7 +8420,7 @@
       <c r="B170" s="2" t="inlineStr"/>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -8469,7 +8469,7 @@
       <c r="B171" s="3" t="inlineStr"/>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -8512,7 +8512,7 @@
       <c r="B172" s="2" t="inlineStr"/>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -8555,7 +8555,7 @@
       <c r="B173" s="3" t="inlineStr"/>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -8598,7 +8598,7 @@
       <c r="B174" s="2" t="inlineStr"/>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -8647,7 +8647,7 @@
       <c r="B175" s="3" t="inlineStr"/>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -8690,7 +8690,7 @@
       <c r="B176" s="2" t="inlineStr"/>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -8739,7 +8739,7 @@
       <c r="B177" s="3" t="inlineStr"/>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -8788,7 +8788,7 @@
       <c r="B178" s="2" t="inlineStr"/>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -8831,7 +8831,7 @@
       <c r="B179" s="3" t="inlineStr"/>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -8874,7 +8874,7 @@
       <c r="B180" s="2" t="inlineStr"/>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -8921,7 +8921,7 @@
       <c r="B181" s="3" t="inlineStr"/>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -8968,7 +8968,7 @@
       <c r="B182" s="2" t="inlineStr"/>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -9007,7 +9007,7 @@
       <c r="B183" s="3" t="inlineStr"/>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -9056,7 +9056,7 @@
       <c r="B184" s="2" t="inlineStr"/>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -9105,7 +9105,7 @@
       <c r="B185" s="3" t="inlineStr"/>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -9154,7 +9154,7 @@
       <c r="B186" s="2" t="inlineStr"/>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -9203,7 +9203,7 @@
       <c r="B187" s="3" t="inlineStr"/>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -9246,7 +9246,7 @@
       <c r="B188" s="2" t="inlineStr"/>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -9289,7 +9289,7 @@
       <c r="B189" s="3" t="inlineStr"/>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -9338,7 +9338,7 @@
       <c r="B190" s="2" t="inlineStr"/>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -9381,7 +9381,7 @@
       <c r="B191" s="3" t="inlineStr"/>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -9424,7 +9424,7 @@
       <c r="B192" s="2" t="inlineStr"/>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -9471,7 +9471,7 @@
       <c r="B193" s="3" t="inlineStr"/>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -9514,7 +9514,7 @@
       <c r="B194" s="2" t="inlineStr"/>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -9561,7 +9561,7 @@
       <c r="B195" s="3" t="inlineStr"/>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -9604,7 +9604,7 @@
       <c r="B196" s="2" t="inlineStr"/>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -9653,7 +9653,7 @@
       <c r="B197" s="3" t="inlineStr"/>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -9696,7 +9696,7 @@
       <c r="B198" s="2" t="inlineStr"/>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -9743,7 +9743,7 @@
       <c r="B199" s="3" t="inlineStr"/>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -9792,7 +9792,7 @@
       <c r="B200" s="2" t="inlineStr"/>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -9835,7 +9835,7 @@
       <c r="B201" s="3" t="inlineStr"/>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -9884,7 +9884,7 @@
       <c r="B202" s="2" t="inlineStr"/>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -9927,7 +9927,7 @@
       <c r="B203" s="3" t="inlineStr"/>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -9972,7 +9972,7 @@
       <c r="B204" s="2" t="inlineStr"/>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -10021,7 +10021,7 @@
       <c r="B205" s="3" t="inlineStr"/>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -10070,7 +10070,7 @@
       <c r="B206" s="2" t="inlineStr"/>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -10119,7 +10119,7 @@
       <c r="B207" s="3" t="inlineStr"/>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -10168,7 +10168,7 @@
       <c r="B208" s="2" t="inlineStr"/>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -10211,7 +10211,7 @@
       <c r="B209" s="3" t="inlineStr"/>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -10260,7 +10260,7 @@
       <c r="B210" s="2" t="inlineStr"/>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -10303,7 +10303,7 @@
       <c r="B211" s="3" t="inlineStr"/>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -10346,7 +10346,7 @@
       <c r="B212" s="2" t="inlineStr"/>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -10389,7 +10389,7 @@
       <c r="B213" s="3" t="inlineStr"/>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -10432,7 +10432,7 @@
       <c r="B214" s="2" t="inlineStr"/>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -10475,7 +10475,7 @@
       <c r="B215" s="3" t="inlineStr"/>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -10518,7 +10518,7 @@
       <c r="B216" s="2" t="inlineStr"/>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -10561,7 +10561,7 @@
       <c r="B217" s="3" t="inlineStr"/>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -10604,7 +10604,7 @@
       <c r="B218" s="2" t="inlineStr"/>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -10653,7 +10653,7 @@
       <c r="B219" s="3" t="inlineStr"/>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -10696,7 +10696,7 @@
       <c r="B220" s="2" t="inlineStr"/>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -10739,7 +10739,7 @@
       <c r="B221" s="3" t="inlineStr"/>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -10782,7 +10782,7 @@
       <c r="B222" s="2" t="inlineStr"/>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -10831,7 +10831,7 @@
       <c r="B223" s="3" t="inlineStr"/>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -10874,7 +10874,7 @@
       <c r="B224" s="2" t="inlineStr"/>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -10923,7 +10923,7 @@
       <c r="B225" s="3" t="inlineStr"/>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -10966,7 +10966,7 @@
       <c r="B226" s="2" t="inlineStr"/>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -11009,7 +11009,7 @@
       <c r="B227" s="3" t="inlineStr"/>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -11052,7 +11052,7 @@
       <c r="B228" s="2" t="inlineStr"/>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -11101,7 +11101,7 @@
       <c r="B229" s="3" t="inlineStr"/>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -11150,7 +11150,7 @@
       <c r="B230" s="2" t="inlineStr"/>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       <c r="B231" s="3" t="inlineStr"/>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -11236,7 +11236,7 @@
       <c r="B232" s="2" t="inlineStr"/>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -11279,7 +11279,7 @@
       <c r="B233" s="3" t="inlineStr"/>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -11328,7 +11328,7 @@
       <c r="B234" s="2" t="inlineStr"/>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -11377,7 +11377,7 @@
       <c r="B235" s="3" t="inlineStr"/>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -11426,7 +11426,7 @@
       <c r="B236" s="2" t="inlineStr"/>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -11471,7 +11471,7 @@
       <c r="B237" s="3" t="inlineStr"/>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -11520,7 +11520,7 @@
       <c r="B238" s="2" t="inlineStr"/>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -11569,7 +11569,7 @@
       <c r="B239" s="3" t="inlineStr"/>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -11618,7 +11618,7 @@
       <c r="B240" s="2" t="inlineStr"/>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -11667,7 +11667,7 @@
       <c r="B241" s="3" t="inlineStr"/>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -11716,7 +11716,7 @@
       <c r="B242" s="2" t="inlineStr"/>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -11759,7 +11759,7 @@
       <c r="B243" s="3" t="inlineStr"/>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -11802,7 +11802,7 @@
       <c r="B244" s="2" t="inlineStr"/>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -11849,7 +11849,7 @@
       <c r="B245" s="3" t="inlineStr"/>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -11894,7 +11894,7 @@
       <c r="B246" s="2" t="inlineStr"/>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -11937,7 +11937,7 @@
       <c r="B247" s="3" t="inlineStr"/>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -11986,7 +11986,7 @@
       <c r="B248" s="2" t="inlineStr"/>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -12029,7 +12029,7 @@
       <c r="B249" s="3" t="inlineStr"/>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -12072,7 +12072,7 @@
       <c r="B250" s="2" t="inlineStr"/>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -12121,7 +12121,7 @@
       <c r="B251" s="3" t="inlineStr"/>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -12164,7 +12164,7 @@
       <c r="B252" s="2" t="inlineStr"/>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -12207,7 +12207,7 @@
       <c r="B253" s="3" t="inlineStr"/>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -12250,7 +12250,7 @@
       <c r="B254" s="2" t="inlineStr"/>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -12299,7 +12299,7 @@
       <c r="B255" s="3" t="inlineStr"/>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -12348,7 +12348,7 @@
       <c r="B256" s="2" t="inlineStr"/>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -12397,7 +12397,7 @@
       <c r="B257" s="3" t="inlineStr"/>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -12440,7 +12440,7 @@
       <c r="B258" s="2" t="inlineStr"/>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -12489,7 +12489,7 @@
       <c r="B259" s="3" t="inlineStr"/>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -12538,7 +12538,7 @@
       <c r="B260" s="2" t="inlineStr"/>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -12581,7 +12581,7 @@
       <c r="B261" s="3" t="inlineStr"/>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -12630,7 +12630,7 @@
       <c r="B262" s="2" t="inlineStr"/>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -12673,7 +12673,7 @@
       <c r="B263" s="3" t="inlineStr"/>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -12722,7 +12722,7 @@
       <c r="B264" s="2" t="inlineStr"/>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -12771,7 +12771,7 @@
       <c r="B265" s="3" t="inlineStr"/>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -12820,7 +12820,7 @@
       <c r="B266" s="2" t="inlineStr"/>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -12869,7 +12869,7 @@
       <c r="B267" s="3" t="inlineStr"/>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -12912,7 +12912,7 @@
       <c r="B268" s="2" t="inlineStr"/>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -12951,7 +12951,7 @@
       <c r="B269" s="3" t="inlineStr"/>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -12994,7 +12994,7 @@
       <c r="B270" s="2" t="inlineStr"/>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -13043,7 +13043,7 @@
       <c r="B271" s="3" t="inlineStr"/>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -13090,7 +13090,7 @@
       <c r="B272" s="2" t="inlineStr"/>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -13133,7 +13133,7 @@
       <c r="B273" s="3" t="inlineStr"/>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -13182,7 +13182,7 @@
       <c r="B274" s="2" t="inlineStr"/>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       <c r="B275" s="3" t="inlineStr"/>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -13274,7 +13274,7 @@
       <c r="B276" s="2" t="inlineStr"/>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -13317,7 +13317,7 @@
       <c r="B277" s="3" t="inlineStr"/>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -13366,7 +13366,7 @@
       <c r="B278" s="2" t="inlineStr"/>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -13415,7 +13415,7 @@
       <c r="B279" s="3" t="inlineStr"/>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -13458,7 +13458,7 @@
       <c r="B280" s="2" t="inlineStr"/>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -13505,7 +13505,7 @@
       <c r="B281" s="3" t="inlineStr"/>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -13554,7 +13554,7 @@
       <c r="B282" s="2" t="inlineStr"/>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -13597,7 +13597,7 @@
       <c r="B283" s="3" t="inlineStr"/>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -13640,7 +13640,7 @@
       <c r="B284" s="2" t="inlineStr"/>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -13689,7 +13689,7 @@
       <c r="B285" s="3" t="inlineStr"/>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -13738,7 +13738,7 @@
       <c r="B286" s="2" t="inlineStr"/>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -13785,7 +13785,7 @@
       <c r="B287" s="3" t="inlineStr"/>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -13828,7 +13828,7 @@
       <c r="B288" s="2" t="inlineStr"/>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -13877,7 +13877,7 @@
       <c r="B289" s="3" t="inlineStr"/>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -13926,7 +13926,7 @@
       <c r="B290" s="2" t="inlineStr"/>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -13975,7 +13975,7 @@
       <c r="B291" s="3" t="inlineStr"/>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -14024,7 +14024,7 @@
       <c r="B292" s="2" t="inlineStr"/>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -14073,7 +14073,7 @@
       <c r="B293" s="3" t="inlineStr"/>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -14122,7 +14122,7 @@
       <c r="B294" s="2" t="inlineStr"/>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -14171,7 +14171,7 @@
       <c r="B295" s="3" t="inlineStr"/>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -14214,7 +14214,7 @@
       <c r="B296" s="2" t="inlineStr"/>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -14263,7 +14263,7 @@
       <c r="B297" s="3" t="inlineStr"/>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -14308,7 +14308,7 @@
       <c r="B298" s="2" t="inlineStr"/>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -14351,7 +14351,7 @@
       <c r="B299" s="3" t="inlineStr"/>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -14394,7 +14394,7 @@
       <c r="B300" s="2" t="inlineStr"/>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -14431,7 +14431,7 @@
       <c r="B301" s="3" t="inlineStr"/>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -14480,7 +14480,7 @@
       <c r="B302" s="2" t="inlineStr"/>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -14527,7 +14527,7 @@
       <c r="B303" s="3" t="inlineStr"/>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -14570,7 +14570,7 @@
       <c r="B304" s="2" t="inlineStr"/>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -14619,7 +14619,7 @@
       <c r="B305" s="3" t="inlineStr"/>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -14662,7 +14662,7 @@
       <c r="B306" s="2" t="inlineStr"/>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -14711,7 +14711,7 @@
       <c r="B307" s="3" t="inlineStr"/>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -14754,7 +14754,7 @@
       <c r="B308" s="2" t="inlineStr"/>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -14797,7 +14797,7 @@
       <c r="B309" s="3" t="inlineStr"/>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -14846,7 +14846,7 @@
       <c r="B310" s="2" t="inlineStr"/>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
@@ -14895,7 +14895,7 @@
       <c r="B311" s="3" t="inlineStr"/>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -14944,7 +14944,7 @@
       <c r="B312" s="2" t="inlineStr"/>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
@@ -14993,7 +14993,7 @@
       <c r="B313" s="3" t="inlineStr"/>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -15040,7 +15040,7 @@
       <c r="B314" s="2" t="inlineStr"/>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -15089,7 +15089,7 @@
       <c r="B315" s="3" t="inlineStr"/>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -15138,7 +15138,7 @@
       <c r="B316" s="2" t="inlineStr"/>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -15187,7 +15187,7 @@
       <c r="B317" s="3" t="inlineStr"/>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -15234,7 +15234,7 @@
       <c r="B318" s="2" t="inlineStr"/>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
@@ -15277,7 +15277,7 @@
       <c r="B319" s="3" t="inlineStr"/>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -15326,7 +15326,7 @@
       <c r="B320" s="2" t="inlineStr"/>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -15373,7 +15373,7 @@
       <c r="B321" s="3" t="inlineStr"/>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -15416,7 +15416,7 @@
       <c r="B322" s="2" t="inlineStr"/>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -15465,7 +15465,7 @@
       <c r="B323" s="3" t="inlineStr"/>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -15508,7 +15508,7 @@
       <c r="B324" s="2" t="inlineStr"/>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -15557,7 +15557,7 @@
       <c r="B325" s="3" t="inlineStr"/>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -15600,7 +15600,7 @@
       <c r="B326" s="2" t="inlineStr"/>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
@@ -15643,7 +15643,7 @@
       <c r="B327" s="3" t="inlineStr"/>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -15690,7 +15690,7 @@
       <c r="B328" s="2" t="inlineStr"/>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
@@ -15739,7 +15739,7 @@
       <c r="B329" s="3" t="inlineStr"/>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -15782,7 +15782,7 @@
       <c r="B330" s="2" t="inlineStr"/>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
@@ -15831,7 +15831,7 @@
       <c r="B331" s="3" t="inlineStr"/>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -15870,7 +15870,7 @@
       <c r="B332" s="2" t="inlineStr"/>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
@@ -15919,7 +15919,7 @@
       <c r="B333" s="3" t="inlineStr"/>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -15962,7 +15962,7 @@
       <c r="B334" s="2" t="inlineStr"/>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
@@ -16011,7 +16011,7 @@
       <c r="B335" s="3" t="inlineStr"/>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -16060,7 +16060,7 @@
       <c r="B336" s="2" t="inlineStr"/>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
@@ -16109,7 +16109,7 @@
       <c r="B337" s="3" t="inlineStr"/>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -16158,7 +16158,7 @@
       <c r="B338" s="2" t="inlineStr"/>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
@@ -16207,7 +16207,7 @@
       <c r="B339" s="3" t="inlineStr"/>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -16256,7 +16256,7 @@
       <c r="B340" s="2" t="inlineStr"/>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
@@ -16305,7 +16305,7 @@
       <c r="B341" s="3" t="inlineStr"/>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -16354,7 +16354,7 @@
       <c r="B342" s="2" t="inlineStr"/>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
@@ -16397,7 +16397,7 @@
       <c r="B343" s="3" t="inlineStr"/>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -16440,7 +16440,7 @@
       <c r="B344" s="2" t="inlineStr"/>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -16489,7 +16489,7 @@
       <c r="B345" s="3" t="inlineStr"/>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -16538,7 +16538,7 @@
       <c r="B346" s="2" t="inlineStr"/>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
@@ -16587,7 +16587,7 @@
       <c r="B347" s="3" t="inlineStr"/>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -16630,7 +16630,7 @@
       <c r="B348" s="2" t="inlineStr"/>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
@@ -16673,7 +16673,7 @@
       <c r="B349" s="3" t="inlineStr"/>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -16722,7 +16722,7 @@
       <c r="B350" s="2" t="inlineStr"/>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -16765,7 +16765,7 @@
       <c r="B351" s="3" t="inlineStr"/>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -16808,7 +16808,7 @@
       <c r="B352" s="2" t="inlineStr"/>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
@@ -16857,7 +16857,7 @@
       <c r="B353" s="3" t="inlineStr"/>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -16906,7 +16906,7 @@
       <c r="B354" s="2" t="inlineStr"/>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -16949,7 +16949,7 @@
       <c r="B355" s="3" t="inlineStr"/>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -16998,7 +16998,7 @@
       <c r="B356" s="2" t="inlineStr"/>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
@@ -17047,7 +17047,7 @@
       <c r="B357" s="3" t="inlineStr"/>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -17096,7 +17096,7 @@
       <c r="B358" s="2" t="inlineStr"/>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
@@ -17143,7 +17143,7 @@
       <c r="B359" s="3" t="inlineStr"/>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -17192,7 +17192,7 @@
       <c r="B360" s="2" t="inlineStr"/>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -17241,7 +17241,7 @@
       <c r="B361" s="3" t="inlineStr"/>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -17284,7 +17284,7 @@
       <c r="B362" s="2" t="inlineStr"/>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
@@ -17333,7 +17333,7 @@
       <c r="B363" s="3" t="inlineStr"/>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -17376,7 +17376,7 @@
       <c r="B364" s="2" t="inlineStr"/>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -17425,7 +17425,7 @@
       <c r="B365" s="3" t="inlineStr"/>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -17474,7 +17474,7 @@
       <c r="B366" s="2" t="inlineStr"/>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
@@ -17517,7 +17517,7 @@
       <c r="B367" s="3" t="inlineStr"/>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -17560,7 +17560,7 @@
       <c r="B368" s="2" t="inlineStr"/>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
@@ -17609,7 +17609,7 @@
       <c r="B369" s="3" t="inlineStr"/>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -17658,7 +17658,7 @@
       <c r="B370" s="2" t="inlineStr"/>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
@@ -17707,7 +17707,7 @@
       <c r="B371" s="3" t="inlineStr"/>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -17750,7 +17750,7 @@
       <c r="B372" s="2" t="inlineStr"/>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
@@ -17789,7 +17789,7 @@
       <c r="B373" s="3" t="inlineStr"/>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -17838,7 +17838,7 @@
       <c r="B374" s="2" t="inlineStr"/>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
@@ -17887,7 +17887,7 @@
       <c r="B375" s="3" t="inlineStr"/>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -17936,7 +17936,7 @@
       <c r="B376" s="2" t="inlineStr"/>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
@@ -17985,7 +17985,7 @@
       <c r="B377" s="3" t="inlineStr"/>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -18028,7 +18028,7 @@
       <c r="B378" s="2" t="inlineStr"/>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
@@ -18077,7 +18077,7 @@
       <c r="B379" s="3" t="inlineStr"/>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -18126,7 +18126,7 @@
       <c r="B380" s="2" t="inlineStr"/>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -18175,7 +18175,7 @@
       <c r="B381" s="3" t="inlineStr"/>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -18224,7 +18224,7 @@
       <c r="B382" s="2" t="inlineStr"/>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -18273,7 +18273,7 @@
       <c r="B383" s="3" t="inlineStr"/>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -18316,7 +18316,7 @@
       <c r="B384" s="2" t="inlineStr"/>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -18359,7 +18359,7 @@
       <c r="B385" s="3" t="inlineStr"/>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -18408,7 +18408,7 @@
       <c r="B386" s="2" t="inlineStr"/>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -18457,7 +18457,7 @@
       <c r="B387" s="3" t="inlineStr"/>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -18500,7 +18500,7 @@
       <c r="B388" s="2" t="inlineStr"/>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
@@ -18549,7 +18549,7 @@
       <c r="B389" s="3" t="inlineStr"/>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -18592,7 +18592,7 @@
       <c r="B390" s="2" t="inlineStr"/>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
@@ -18635,7 +18635,7 @@
       <c r="B391" s="3" t="inlineStr"/>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -18684,7 +18684,7 @@
       <c r="B392" s="2" t="inlineStr"/>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -18733,7 +18733,7 @@
       <c r="B393" s="3" t="inlineStr"/>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D393" s="3" t="inlineStr">
@@ -18782,7 +18782,7 @@
       <c r="B394" s="2" t="inlineStr"/>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
@@ -18825,7 +18825,7 @@
       <c r="B395" s="3" t="inlineStr"/>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D395" s="3" t="inlineStr">
@@ -18874,7 +18874,7 @@
       <c r="B396" s="2" t="inlineStr"/>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
@@ -18917,7 +18917,7 @@
       <c r="B397" s="3" t="inlineStr"/>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D397" s="3" t="inlineStr">
@@ -18966,7 +18966,7 @@
       <c r="B398" s="2" t="inlineStr"/>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
@@ -19005,7 +19005,7 @@
       <c r="B399" s="3" t="inlineStr"/>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D399" s="3" t="inlineStr">
@@ -19054,7 +19054,7 @@
       <c r="B400" s="2" t="inlineStr"/>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
@@ -19101,7 +19101,7 @@
       <c r="B401" s="3" t="inlineStr"/>
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D401" s="3" t="inlineStr">
@@ -19144,7 +19144,7 @@
       <c r="B402" s="2" t="inlineStr"/>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -19193,7 +19193,7 @@
       <c r="B403" s="3" t="inlineStr"/>
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D403" s="3" t="inlineStr">
@@ -19242,7 +19242,7 @@
       <c r="B404" s="2" t="inlineStr"/>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
@@ -19285,7 +19285,7 @@
       <c r="B405" s="3" t="inlineStr"/>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D405" s="3" t="inlineStr">
@@ -19334,7 +19334,7 @@
       <c r="B406" s="2" t="inlineStr"/>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
@@ -19383,7 +19383,7 @@
       <c r="B407" s="3" t="inlineStr"/>
       <c r="C407" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D407" s="3" t="inlineStr">
@@ -19430,7 +19430,7 @@
       <c r="B408" s="2" t="inlineStr"/>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
@@ -19479,7 +19479,7 @@
       <c r="B409" s="3" t="inlineStr"/>
       <c r="C409" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D409" s="3" t="inlineStr">
@@ -19522,7 +19522,7 @@
       <c r="B410" s="2" t="inlineStr"/>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D410" s="2" t="inlineStr">
@@ -19571,7 +19571,7 @@
       <c r="B411" s="3" t="inlineStr"/>
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D411" s="3" t="inlineStr">
@@ -19614,7 +19614,7 @@
       <c r="B412" s="2" t="inlineStr"/>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
@@ -19657,7 +19657,7 @@
       <c r="B413" s="3" t="inlineStr"/>
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D413" s="3" t="inlineStr">
@@ -19692,7 +19692,7 @@
       <c r="B414" s="2" t="inlineStr"/>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
@@ -19741,7 +19741,7 @@
       <c r="B415" s="3" t="inlineStr"/>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D415" s="3" t="inlineStr">
@@ -19790,7 +19790,7 @@
       <c r="B416" s="2" t="inlineStr"/>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
@@ -19837,7 +19837,7 @@
       <c r="B417" s="3" t="inlineStr"/>
       <c r="C417" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D417" s="3" t="inlineStr">
@@ -19886,7 +19886,7 @@
       <c r="B418" s="2" t="inlineStr"/>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
@@ -19929,7 +19929,7 @@
       <c r="B419" s="3" t="inlineStr"/>
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D419" s="3" t="inlineStr">
@@ -19972,7 +19972,7 @@
       <c r="B420" s="2" t="inlineStr"/>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
@@ -20021,7 +20021,7 @@
       <c r="B421" s="3" t="inlineStr"/>
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D421" s="3" t="inlineStr">
@@ -20070,7 +20070,7 @@
       <c r="B422" s="2" t="inlineStr"/>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
@@ -20113,7 +20113,7 @@
       <c r="B423" s="3" t="inlineStr"/>
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D423" s="3" t="inlineStr">
@@ -20162,7 +20162,7 @@
       <c r="B424" s="2" t="inlineStr"/>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
@@ -20205,7 +20205,7 @@
       <c r="B425" s="3" t="inlineStr"/>
       <c r="C425" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D425" s="3" t="inlineStr">
@@ -20248,7 +20248,7 @@
       <c r="B426" s="2" t="inlineStr"/>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
@@ -20291,7 +20291,7 @@
       <c r="B427" s="3" t="inlineStr"/>
       <c r="C427" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D427" s="3" t="inlineStr">
@@ -20334,7 +20334,7 @@
       <c r="B428" s="2" t="inlineStr"/>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
@@ -20383,7 +20383,7 @@
       <c r="B429" s="3" t="inlineStr"/>
       <c r="C429" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D429" s="3" t="inlineStr">
@@ -20432,7 +20432,7 @@
       <c r="B430" s="2" t="inlineStr"/>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -20481,7 +20481,7 @@
       <c r="B431" s="3" t="inlineStr"/>
       <c r="C431" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D431" s="3" t="inlineStr">
@@ -20530,7 +20530,7 @@
       <c r="B432" s="2" t="inlineStr"/>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
@@ -20573,7 +20573,7 @@
       <c r="B433" s="3" t="inlineStr"/>
       <c r="C433" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D433" s="3" t="inlineStr">
@@ -20622,7 +20622,7 @@
       <c r="B434" s="2" t="inlineStr"/>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
@@ -20671,7 +20671,7 @@
       <c r="B435" s="3" t="inlineStr"/>
       <c r="C435" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D435" s="3" t="inlineStr">
@@ -20720,7 +20720,7 @@
       <c r="B436" s="2" t="inlineStr"/>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
@@ -20769,7 +20769,7 @@
       <c r="B437" s="3" t="inlineStr"/>
       <c r="C437" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D437" s="3" t="inlineStr">
@@ -20814,7 +20814,7 @@
       <c r="B438" s="2" t="inlineStr"/>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
@@ -20857,7 +20857,7 @@
       <c r="B439" s="3" t="inlineStr"/>
       <c r="C439" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D439" s="3" t="inlineStr">
@@ -20902,7 +20902,7 @@
       <c r="B440" s="2" t="inlineStr"/>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D440" s="2" t="inlineStr">
@@ -20951,7 +20951,7 @@
       <c r="B441" s="3" t="inlineStr"/>
       <c r="C441" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D441" s="3" t="inlineStr">
@@ -21000,7 +21000,7 @@
       <c r="B442" s="2" t="inlineStr"/>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
@@ -21045,7 +21045,7 @@
       <c r="B443" s="3" t="inlineStr"/>
       <c r="C443" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D443" s="3" t="inlineStr">
@@ -21094,7 +21094,7 @@
       <c r="B444" s="2" t="inlineStr"/>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -21143,7 +21143,7 @@
       <c r="B445" s="3" t="inlineStr"/>
       <c r="C445" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D445" s="3" t="inlineStr">
@@ -21192,7 +21192,7 @@
       <c r="B446" s="2" t="inlineStr"/>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
@@ -21241,7 +21241,7 @@
       <c r="B447" s="3" t="inlineStr"/>
       <c r="C447" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D447" s="3" t="inlineStr">
@@ -21284,7 +21284,7 @@
       <c r="B448" s="2" t="inlineStr"/>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
@@ -21327,7 +21327,7 @@
       <c r="B449" s="3" t="inlineStr"/>
       <c r="C449" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D449" s="3" t="inlineStr">
@@ -21370,7 +21370,7 @@
       <c r="B450" s="2" t="inlineStr"/>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
@@ -21417,7 +21417,7 @@
       <c r="B451" s="3" t="inlineStr"/>
       <c r="C451" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D451" s="3" t="inlineStr">
@@ -21462,7 +21462,7 @@
       <c r="B452" s="2" t="inlineStr"/>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
@@ -21511,7 +21511,7 @@
       <c r="B453" s="3" t="inlineStr"/>
       <c r="C453" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D453" s="3" t="inlineStr">
@@ -21554,7 +21554,7 @@
       <c r="B454" s="2" t="inlineStr"/>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
@@ -21593,7 +21593,7 @@
       <c r="B455" s="3" t="inlineStr"/>
       <c r="C455" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D455" s="3" t="inlineStr">
@@ -21642,7 +21642,7 @@
       <c r="B456" s="2" t="inlineStr"/>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -21685,7 +21685,7 @@
       <c r="B457" s="3" t="inlineStr"/>
       <c r="C457" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D457" s="3" t="inlineStr">
@@ -21734,7 +21734,7 @@
       <c r="B458" s="2" t="inlineStr"/>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
@@ -21783,7 +21783,7 @@
       <c r="B459" s="3" t="inlineStr"/>
       <c r="C459" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D459" s="3" t="inlineStr">
@@ -21832,7 +21832,7 @@
       <c r="B460" s="2" t="inlineStr"/>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
@@ -21875,7 +21875,7 @@
       <c r="B461" s="3" t="inlineStr"/>
       <c r="C461" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D461" s="3" t="inlineStr">
@@ -21924,7 +21924,7 @@
       <c r="B462" s="2" t="inlineStr"/>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
@@ -21973,7 +21973,7 @@
       <c r="B463" s="3" t="inlineStr"/>
       <c r="C463" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D463" s="3" t="inlineStr">
@@ -22022,7 +22022,7 @@
       <c r="B464" s="2" t="inlineStr"/>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -22065,7 +22065,7 @@
       <c r="B465" s="3" t="inlineStr"/>
       <c r="C465" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D465" s="3" t="inlineStr">
@@ -22114,7 +22114,7 @@
       <c r="B466" s="2" t="inlineStr"/>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -22163,7 +22163,7 @@
       <c r="B467" s="3" t="inlineStr"/>
       <c r="C467" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D467" s="3" t="inlineStr">
@@ -22206,7 +22206,7 @@
       <c r="B468" s="2" t="inlineStr"/>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D468" s="2" t="inlineStr">
@@ -22255,7 +22255,7 @@
       <c r="B469" s="3" t="inlineStr"/>
       <c r="C469" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D469" s="3" t="inlineStr">
@@ -22298,7 +22298,7 @@
       <c r="B470" s="2" t="inlineStr"/>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D470" s="2" t="inlineStr">
@@ -22347,7 +22347,7 @@
       <c r="B471" s="3" t="inlineStr"/>
       <c r="C471" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D471" s="3" t="inlineStr">
@@ -22396,7 +22396,7 @@
       <c r="B472" s="2" t="inlineStr"/>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D472" s="2" t="inlineStr">
@@ -22445,7 +22445,7 @@
       <c r="B473" s="3" t="inlineStr"/>
       <c r="C473" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D473" s="3" t="inlineStr">
@@ -22488,7 +22488,7 @@
       <c r="B474" s="2" t="inlineStr"/>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
@@ -22537,7 +22537,7 @@
       <c r="B475" s="3" t="inlineStr"/>
       <c r="C475" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D475" s="3" t="inlineStr">
@@ -22580,7 +22580,7 @@
       <c r="B476" s="2" t="inlineStr"/>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
@@ -22623,7 +22623,7 @@
       <c r="B477" s="3" t="inlineStr"/>
       <c r="C477" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D477" s="3" t="inlineStr">
@@ -22666,7 +22666,7 @@
       <c r="B478" s="2" t="inlineStr"/>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -22709,7 +22709,7 @@
       <c r="B479" s="3" t="inlineStr"/>
       <c r="C479" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D479" s="3" t="inlineStr">
@@ -22758,7 +22758,7 @@
       <c r="B480" s="2" t="inlineStr"/>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
@@ -22807,7 +22807,7 @@
       <c r="B481" s="3" t="inlineStr"/>
       <c r="C481" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D481" s="3" t="inlineStr">
@@ -22850,7 +22850,7 @@
       <c r="B482" s="2" t="inlineStr"/>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
@@ -22899,7 +22899,7 @@
       <c r="B483" s="3" t="inlineStr"/>
       <c r="C483" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D483" s="3" t="inlineStr">
@@ -22942,7 +22942,7 @@
       <c r="B484" s="2" t="inlineStr"/>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -22991,7 +22991,7 @@
       <c r="B485" s="3" t="inlineStr"/>
       <c r="C485" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D485" s="3" t="inlineStr">
@@ -23040,7 +23040,7 @@
       <c r="B486" s="2" t="inlineStr"/>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -23089,7 +23089,7 @@
       <c r="B487" s="3" t="inlineStr"/>
       <c r="C487" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D487" s="3" t="inlineStr">
@@ -23138,7 +23138,7 @@
       <c r="B488" s="2" t="inlineStr"/>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -23181,7 +23181,7 @@
       <c r="B489" s="3" t="inlineStr"/>
       <c r="C489" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D489" s="3" t="inlineStr">
@@ -23224,7 +23224,7 @@
       <c r="B490" s="2" t="inlineStr"/>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -23269,7 +23269,7 @@
       <c r="B491" s="3" t="inlineStr"/>
       <c r="C491" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D491" s="3" t="inlineStr">
@@ -23318,7 +23318,7 @@
       <c r="B492" s="2" t="inlineStr"/>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -23367,7 +23367,7 @@
       <c r="B493" s="3" t="inlineStr"/>
       <c r="C493" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D493" s="3" t="inlineStr">
@@ -23416,7 +23416,7 @@
       <c r="B494" s="2" t="inlineStr"/>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -23461,7 +23461,7 @@
       <c r="B495" s="3" t="inlineStr"/>
       <c r="C495" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D495" s="3" t="inlineStr">
@@ -23504,7 +23504,7 @@
       <c r="B496" s="2" t="inlineStr"/>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D496" s="2" t="inlineStr">
@@ -23553,7 +23553,7 @@
       <c r="B497" s="3" t="inlineStr"/>
       <c r="C497" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D497" s="3" t="inlineStr">
@@ -23596,7 +23596,7 @@
       <c r="B498" s="2" t="inlineStr"/>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -23639,7 +23639,7 @@
       <c r="B499" s="3" t="inlineStr"/>
       <c r="C499" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D499" s="3" t="inlineStr">
@@ -23688,7 +23688,7 @@
       <c r="B500" s="2" t="inlineStr"/>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D500" s="2" t="inlineStr">
@@ -23731,7 +23731,7 @@
       <c r="B501" s="3" t="inlineStr"/>
       <c r="C501" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D501" s="3" t="inlineStr">
@@ -23780,7 +23780,7 @@
       <c r="B502" s="2" t="inlineStr"/>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
@@ -23823,7 +23823,7 @@
       <c r="B503" s="3" t="inlineStr"/>
       <c r="C503" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D503" s="3" t="inlineStr">

</xml_diff>